<commit_message>
feat: show inspection deadlines on the briefing and the Fristen page
Counts open the same rows, and HU, UVV and licence dates can be entered and imported.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/import-beispiel.xlsx
+++ b/apps/web/public/import-beispiel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Kennzeichen</t>
   </si>
@@ -25,6 +25,12 @@
     <t>Depot</t>
   </si>
   <si>
+    <t>HU</t>
+  </si>
+  <si>
+    <t>UVV</t>
+  </si>
+  <si>
     <t>K-XLS 1001</t>
   </si>
   <si>
@@ -37,6 +43,12 @@
     <t>Hof Nord</t>
   </si>
   <si>
+    <t>15.06.2027</t>
+  </si>
+  <si>
+    <t>01.09.2026</t>
+  </si>
+  <si>
     <t>K-XLS 1002</t>
   </si>
   <si>
@@ -46,6 +58,12 @@
     <t>Standby</t>
   </si>
   <si>
+    <t>01.03.2026</t>
+  </si>
+  <si>
+    <t>15.11.2026</t>
+  </si>
+  <si>
     <t>K-XLS 1003</t>
   </si>
   <si>
@@ -55,22 +73,40 @@
     <t>Feierabend</t>
   </si>
   <si>
+    <t>30.11.2027</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>K-XLS 1004</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Kein Signal</t>
   </si>
   <si>
     <t>Name</t>
   </si>
   <si>
+    <t>Führerschein gültig bis</t>
+  </si>
+  <si>
+    <t>Führerschein kontrolliert am</t>
+  </si>
+  <si>
     <t>Nora Weber</t>
   </si>
   <si>
+    <t>15.06.2028</t>
+  </si>
+  <si>
+    <t>01.04.2026</t>
+  </si>
+  <si>
     <t>Leo Krüger</t>
+  </si>
+  <si>
+    <t>01.01.2026</t>
   </si>
   <si>
     <t>Fahrer</t>
@@ -94,61 +130,91 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -160,17 +226,35 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -182,7 +266,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -190,26 +274,26 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -221,7 +305,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -229,10 +313,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>